<commit_message>
chore: Box Init함수 구현
생성될 타입 추가 및 아이템 리스트, 레어도 리스트 초기화 함수 추가 및 Init함수에 추가
상자에서 나올 레어도를 정한 후 실제 나올 아이템(레어도에 맞는) 리스트 할당 함수 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/InteractableObject.xlsx
+++ b/JsonConverter/ExcelFiles/InteractableObject.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\JewelThief\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F63B687-05D7-4C58-B357-4520AEF010CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6636F33-9F50-4631-853A-5C06983BC6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29730" yWindow="2625" windowWidth="22485" windowHeight="12495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4500" yWindow="1635" windowWidth="22485" windowHeight="12495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시트1" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,6 @@
  추후 아이템 데이터 Id가 담길 예정</t>
   </si>
   <si>
-    <t>가중치 리스트
- 활률(R,E,U,L)</t>
-  </si>
-  <si>
     <t>Mesh 프리팹 경로</t>
   </si>
   <si>
@@ -140,6 +136,12 @@
   </si>
   <si>
     <t>Object_05</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>확률 리스트
+ 활률(R,E,U,L)
+확률의 총 합이 100을 넘으면 안됨</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -355,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -375,6 +377,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -603,7 +608,7 @@
     <col min="7" max="7" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" ht="36" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -619,162 +624,163 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>16</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="12" t="s">
         <v>20</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>21</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="C5" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>25</v>
-      </c>
       <c r="D5" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="17" t="s">
         <v>26</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="C6" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D6" s="12" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>31</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="17"/>
       <c r="G6" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>